<commit_message>
data: opdater Foedselsdage og jubi.xlsx
</commit_message>
<xml_diff>
--- a/data/Foedselsdage og jubi.xlsx
+++ b/data/Foedselsdage og jubi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KlausVestermark\GitHub\dashboard-hm-sp\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hallmonitordk-my.sharepoint.com/personal/klaus_hallmonitor_dk/Documents/Dokumenter/GitHub/dashboard-hm-sp-backup/dashboard-hm-sp/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{95F85DD0-E6A4-41FC-9618-64CF28A736EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{95F85DD0-E6A4-41FC-9618-64CF28A736EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67B5F2E1-09CB-4A6F-9EB1-BA78B5AE3A81}"/>
   <bookViews>
-    <workbookView xWindow="24480" yWindow="2730" windowWidth="18690" windowHeight="18720" xr2:uid="{471D20D5-FD9F-4E7C-94CA-267ECDE0AE3F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{471D20D5-FD9F-4E7C-94CA-267ECDE0AE3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>DATAPILOTS</t>
   </si>
@@ -129,6 +129,12 @@
   </si>
   <si>
     <t>Søren Lose</t>
+  </si>
+  <si>
+    <t>Torben Bak</t>
+  </si>
+  <si>
+    <t>Joen Olsen</t>
   </si>
 </sst>
 </file>
@@ -212,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -223,29 +229,23 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -582,7 +582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDA4BBF6-BAA1-4BC6-8F75-2F3C17956DDB}">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.28515625" customWidth="1"/>
@@ -591,10 +591,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
+      <c r="B1" s="6"/>
       <c r="C1" t="s">
         <v>23</v>
       </c>
@@ -603,178 +603,192 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="11">
+      <c r="B2" s="8"/>
+      <c r="C2" s="4">
         <v>29051</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="4">
         <v>39630</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="4">
+        <v>35262</v>
+      </c>
+      <c r="D3" s="4">
+        <v>46054</v>
+      </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="11">
+      <c r="B4" s="8"/>
+      <c r="C4" s="4">
         <v>35901</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="4">
         <v>44896</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="11">
+      <c r="B5" s="8"/>
+      <c r="C5" s="4">
         <v>35445</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="4">
         <v>45103</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="4">
         <v>36270</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="4">
         <v>45870</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="5"/>
+      <c r="B7" s="6"/>
     </row>
     <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="11">
+      <c r="B8" s="8"/>
+      <c r="C8" s="4">
         <v>28307</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>44256</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="11">
+      <c r="B9" s="8"/>
+      <c r="C9" s="4">
         <v>31195</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="4">
         <v>44874</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="6"/>
-      <c r="B10" s="7"/>
+      <c r="A10" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="4">
+        <v>29795</v>
+      </c>
+      <c r="D10" s="4">
+        <v>46097</v>
+      </c>
     </row>
     <row r="11" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="5"/>
+      <c r="B11" s="6"/>
     </row>
     <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="11">
+      <c r="B12" s="8"/>
+      <c r="C12" s="4">
         <v>25297</v>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="4">
         <v>45153</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="11">
+      <c r="B13" s="8"/>
+      <c r="C13" s="4">
         <v>29573</v>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="4">
         <v>46054</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="11">
+      <c r="B14" s="8"/>
+      <c r="C14" s="4">
         <v>30807</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="4">
         <v>45691</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="6"/>
-      <c r="B15" s="7"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="8"/>
     </row>
     <row r="16" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="5"/>
+      <c r="B16" s="6"/>
     </row>
     <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="11">
+      <c r="B17" s="8"/>
+      <c r="C17" s="4">
         <v>31134</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="4">
         <v>45231</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="11">
+      <c r="B18" s="8"/>
+      <c r="C18" s="4">
         <v>34547</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="4">
         <v>45566</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="11">
+      <c r="B19" s="8"/>
+      <c r="C19" s="4">
         <v>31587</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="4">
         <v>44564</v>
       </c>
     </row>
@@ -783,10 +797,10 @@
       <c r="B20" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="4">
         <v>36394</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="4">
         <v>45200</v>
       </c>
     </row>
@@ -795,10 +809,10 @@
       <c r="B21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="4">
         <v>35730</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="4">
         <v>45957</v>
       </c>
     </row>
@@ -807,10 +821,10 @@
       <c r="B22" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="4">
         <v>34755</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="4">
         <v>44047</v>
       </c>
     </row>
@@ -819,10 +833,10 @@
       <c r="B23" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="4">
         <v>32403</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="4">
         <v>44287</v>
       </c>
     </row>
@@ -831,10 +845,10 @@
       <c r="B24" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="4">
         <v>39481</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="4">
         <v>45223</v>
       </c>
     </row>
@@ -843,33 +857,33 @@
       <c r="B25" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="4">
         <v>38845</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="4">
         <v>45223</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="11">
+      <c r="B26" s="10"/>
+      <c r="C26" s="4">
         <v>33057</v>
       </c>
-      <c r="D26" s="11">
+      <c r="D26" s="4">
         <v>41275</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B27" s="12" t="s">
+      <c r="B27" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="4">
         <v>40589</v>
       </c>
-      <c r="D27" s="11">
+      <c r="D27" s="4">
         <v>45516</v>
       </c>
     </row>
@@ -877,21 +891,21 @@
       <c r="B28" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="11">
+      <c r="C28" s="4">
         <v>29478</v>
       </c>
-      <c r="D28" s="11">
+      <c r="D28" s="4">
         <v>45658</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B29" s="12" t="s">
+      <c r="B29" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="4">
         <v>39485</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="4">
         <v>46054</v>
       </c>
     </row>
@@ -899,10 +913,10 @@
       <c r="B30" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="4">
         <v>40632</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="4">
         <v>45589</v>
       </c>
     </row>
@@ -910,25 +924,26 @@
       <c r="B31" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="4">
         <v>29820</v>
       </c>
-      <c r="D31" s="11">
+      <c r="D31" s="4">
         <v>43882</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B32" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32" s="4">
+        <v>31772</v>
+      </c>
+      <c r="D32" s="4">
+        <v>46181</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A10:B10"/>
@@ -938,6 +953,16 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A26:B26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data: opdater Foedselsdage og jubi.xlsx (#10)
</commit_message>
<xml_diff>
--- a/data/Foedselsdage og jubi.xlsx
+++ b/data/Foedselsdage og jubi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KlausVestermark\GitHub\dashboard-hm-sp\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hallmonitordk-my.sharepoint.com/personal/klaus_hallmonitor_dk/Documents/Dokumenter/GitHub/dashboard-hm-sp-backup/dashboard-hm-sp/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{95F85DD0-E6A4-41FC-9618-64CF28A736EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{95F85DD0-E6A4-41FC-9618-64CF28A736EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67B5F2E1-09CB-4A6F-9EB1-BA78B5AE3A81}"/>
   <bookViews>
-    <workbookView xWindow="24480" yWindow="2730" windowWidth="18690" windowHeight="18720" xr2:uid="{471D20D5-FD9F-4E7C-94CA-267ECDE0AE3F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{471D20D5-FD9F-4E7C-94CA-267ECDE0AE3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>DATAPILOTS</t>
   </si>
@@ -129,6 +129,12 @@
   </si>
   <si>
     <t>Søren Lose</t>
+  </si>
+  <si>
+    <t>Torben Bak</t>
+  </si>
+  <si>
+    <t>Joen Olsen</t>
   </si>
 </sst>
 </file>
@@ -212,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -223,29 +229,23 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -582,7 +582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDA4BBF6-BAA1-4BC6-8F75-2F3C17956DDB}">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.28515625" customWidth="1"/>
@@ -591,10 +591,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
+      <c r="B1" s="6"/>
       <c r="C1" t="s">
         <v>23</v>
       </c>
@@ -603,178 +603,192 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="11">
+      <c r="B2" s="8"/>
+      <c r="C2" s="4">
         <v>29051</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="4">
         <v>39630</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="4">
+        <v>35262</v>
+      </c>
+      <c r="D3" s="4">
+        <v>46054</v>
+      </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="11">
+      <c r="B4" s="8"/>
+      <c r="C4" s="4">
         <v>35901</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="4">
         <v>44896</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="11">
+      <c r="B5" s="8"/>
+      <c r="C5" s="4">
         <v>35445</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="4">
         <v>45103</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="4">
         <v>36270</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="4">
         <v>45870</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="5"/>
+      <c r="B7" s="6"/>
     </row>
     <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="11">
+      <c r="B8" s="8"/>
+      <c r="C8" s="4">
         <v>28307</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="4">
         <v>44256</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="11">
+      <c r="B9" s="8"/>
+      <c r="C9" s="4">
         <v>31195</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="4">
         <v>44874</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="6"/>
-      <c r="B10" s="7"/>
+      <c r="A10" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="4">
+        <v>29795</v>
+      </c>
+      <c r="D10" s="4">
+        <v>46097</v>
+      </c>
     </row>
     <row r="11" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="5"/>
+      <c r="B11" s="6"/>
     </row>
     <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="11">
+      <c r="B12" s="8"/>
+      <c r="C12" s="4">
         <v>25297</v>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="4">
         <v>45153</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="11">
+      <c r="B13" s="8"/>
+      <c r="C13" s="4">
         <v>29573</v>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="4">
         <v>46054</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="11">
+      <c r="B14" s="8"/>
+      <c r="C14" s="4">
         <v>30807</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="4">
         <v>45691</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="6"/>
-      <c r="B15" s="7"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="8"/>
     </row>
     <row r="16" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="5"/>
+      <c r="B16" s="6"/>
     </row>
     <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="11">
+      <c r="B17" s="8"/>
+      <c r="C17" s="4">
         <v>31134</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="4">
         <v>45231</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="11">
+      <c r="B18" s="8"/>
+      <c r="C18" s="4">
         <v>34547</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="4">
         <v>45566</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="11">
+      <c r="B19" s="8"/>
+      <c r="C19" s="4">
         <v>31587</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="4">
         <v>44564</v>
       </c>
     </row>
@@ -783,10 +797,10 @@
       <c r="B20" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="4">
         <v>36394</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="4">
         <v>45200</v>
       </c>
     </row>
@@ -795,10 +809,10 @@
       <c r="B21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="4">
         <v>35730</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="4">
         <v>45957</v>
       </c>
     </row>
@@ -807,10 +821,10 @@
       <c r="B22" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="4">
         <v>34755</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="4">
         <v>44047</v>
       </c>
     </row>
@@ -819,10 +833,10 @@
       <c r="B23" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="4">
         <v>32403</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="4">
         <v>44287</v>
       </c>
     </row>
@@ -831,10 +845,10 @@
       <c r="B24" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="4">
         <v>39481</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="4">
         <v>45223</v>
       </c>
     </row>
@@ -843,33 +857,33 @@
       <c r="B25" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="4">
         <v>38845</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="4">
         <v>45223</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="11">
+      <c r="B26" s="10"/>
+      <c r="C26" s="4">
         <v>33057</v>
       </c>
-      <c r="D26" s="11">
+      <c r="D26" s="4">
         <v>41275</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B27" s="12" t="s">
+      <c r="B27" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="4">
         <v>40589</v>
       </c>
-      <c r="D27" s="11">
+      <c r="D27" s="4">
         <v>45516</v>
       </c>
     </row>
@@ -877,21 +891,21 @@
       <c r="B28" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="11">
+      <c r="C28" s="4">
         <v>29478</v>
       </c>
-      <c r="D28" s="11">
+      <c r="D28" s="4">
         <v>45658</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B29" s="12" t="s">
+      <c r="B29" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="4">
         <v>39485</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="4">
         <v>46054</v>
       </c>
     </row>
@@ -899,10 +913,10 @@
       <c r="B30" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="4">
         <v>40632</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="4">
         <v>45589</v>
       </c>
     </row>
@@ -910,25 +924,26 @@
       <c r="B31" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="4">
         <v>29820</v>
       </c>
-      <c r="D31" s="11">
+      <c r="D31" s="4">
         <v>43882</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B32" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32" s="4">
+        <v>31772</v>
+      </c>
+      <c r="D32" s="4">
+        <v>46181</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A10:B10"/>
@@ -938,6 +953,16 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A26:B26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data: ret Marcos fødselsår fra 1977 til 1976
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Foedselsdage og jubi.xlsx
+++ b/data/Foedselsdage og jubi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hallmonitordk-my.sharepoint.com/personal/klaus_hallmonitor_dk/Documents/Dokumenter/GitHub/dashboard-hm-sp-backup/dashboard-hm-sp/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{95F85DD0-E6A4-41FC-9618-64CF28A736EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67B5F2E1-09CB-4A6F-9EB1-BA78B5AE3A81}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{95F85DD0-E6A4-41FC-9618-64CF28A736EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D992646E-9726-438E-BD2D-A131E981F1C6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{471D20D5-FD9F-4E7C-94CA-267ECDE0AE3F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{471D20D5-FD9F-4E7C-94CA-267ECDE0AE3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -230,17 +230,17 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -591,10 +591,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
+      <c r="B1" s="8"/>
       <c r="C1" t="s">
         <v>23</v>
       </c>
@@ -603,10 +603,10 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="8"/>
+      <c r="B2" s="6"/>
       <c r="C2" s="4">
         <v>29051</v>
       </c>
@@ -615,10 +615,10 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8"/>
+      <c r="B3" s="6"/>
       <c r="C3" s="4">
         <v>35262</v>
       </c>
@@ -627,10 +627,10 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="8"/>
+      <c r="B4" s="6"/>
       <c r="C4" s="4">
         <v>35901</v>
       </c>
@@ -639,10 +639,10 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="8"/>
+      <c r="B5" s="6"/>
       <c r="C5" s="4">
         <v>35445</v>
       </c>
@@ -663,28 +663,28 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="6"/>
+      <c r="B7" s="8"/>
     </row>
     <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="8"/>
+      <c r="B8" s="6"/>
       <c r="C8" s="4">
-        <v>28307</v>
+        <v>27942</v>
       </c>
       <c r="D8" s="4">
         <v>44256</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="8"/>
+      <c r="B9" s="6"/>
       <c r="C9" s="4">
         <v>31195</v>
       </c>
@@ -693,10 +693,10 @@
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="8"/>
+      <c r="B10" s="6"/>
       <c r="C10" s="4">
         <v>29795</v>
       </c>
@@ -705,16 +705,16 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="6"/>
+      <c r="B11" s="8"/>
     </row>
     <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="8"/>
+      <c r="B12" s="6"/>
       <c r="C12" s="4">
         <v>25297</v>
       </c>
@@ -723,10 +723,10 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="8"/>
+      <c r="B13" s="6"/>
       <c r="C13" s="4">
         <v>29573</v>
       </c>
@@ -735,10 +735,10 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="8"/>
+      <c r="B14" s="6"/>
       <c r="C14" s="4">
         <v>30807</v>
       </c>
@@ -747,20 +747,20 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="8"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="6"/>
     </row>
     <row r="16" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="6"/>
+      <c r="B16" s="8"/>
     </row>
     <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="8"/>
+      <c r="B17" s="6"/>
       <c r="C17" s="4">
         <v>31134</v>
       </c>
@@ -769,10 +769,10 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="8"/>
+      <c r="B18" s="6"/>
       <c r="C18" s="4">
         <v>34547</v>
       </c>
@@ -781,10 +781,10 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="8"/>
+      <c r="B19" s="6"/>
       <c r="C19" s="4">
         <v>31587</v>
       </c>
@@ -944,6 +944,16 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A10:B10"/>
@@ -953,16 +963,6 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A26:B26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>